<commit_message>
Udating test-data and correcting 5-equations system
</commit_message>
<xml_diff>
--- a/Tests Data/CanadianSolar CS6P-250P/Single-diode model/G = 765 W.m^-2 and T = 44.5 ºC/Single-diode emulator - CanadianSolar CS6P-250P (ref = STC, G = 765 and T = 44.5).xlsx
+++ b/Tests Data/CanadianSolar CS6P-250P/Single-diode model/G = 765 W.m^-2 and T = 44.5 ºC/Single-diode emulator - CanadianSolar CS6P-250P (ref = STC, G = 765 and T = 44.5).xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Gabriel\Desktop\Stage_GeePs\Test Data - new\CanadianSolar CS6P-250P\Single-diode model\S = 765 W.m^-2 and T = 44.5 ºC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Gabriel\Desktop\Stage_GeePs\PV-emulator\Tests Data\CanadianSolar CS6P-250P\Single-diode model\G = 765 W.m^-2 and T = 44.5 ºC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BF75DF1-4700-4E98-9C6B-E140EF7D32BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B49BC9F-75EB-4BF7-9B1F-0725037D276D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10140" yWindow="0" windowWidth="10455" windowHeight="10905" xr2:uid="{217CCB4B-160F-4504-987F-9C10DFEEC66E}"/>
+    <workbookView xWindow="30570" yWindow="0" windowWidth="18825" windowHeight="15585" xr2:uid="{217CCB4B-160F-4504-987F-9C10DFEEC66E}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -537,57 +537,57 @@
         <v>60</v>
       </c>
       <c r="B2">
-        <v>2.42</v>
+        <v>2.75</v>
       </c>
       <c r="C2">
         <f>A2*B2</f>
-        <v>145.19999999999999</v>
+        <v>165</v>
       </c>
       <c r="D2">
-        <v>19.600000000000001</v>
+        <v>22.24</v>
       </c>
       <c r="E2">
-        <v>6.78</v>
+        <v>6.82</v>
       </c>
       <c r="F2">
         <f>D2*E2</f>
-        <v>132.88800000000001</v>
+        <v>151.67679999999999</v>
       </c>
       <c r="G2">
         <f>D2/E2</f>
-        <v>2.8908554572271385</v>
+        <v>3.2609970674486801</v>
       </c>
       <c r="H2">
-        <v>35.784858999999997</v>
+        <v>36.470618999999999</v>
       </c>
       <c r="I2">
-        <v>12.165794</v>
+        <v>10.97875</v>
       </c>
       <c r="J2">
-        <v>20.089265999999999</v>
+        <v>22.642405</v>
       </c>
       <c r="K2">
-        <v>6.8297569999999999</v>
+        <v>6.8160420000000004</v>
       </c>
       <c r="L2">
         <f>J2/K2</f>
-        <v>2.9414320304514492</v>
+        <v>3.3219286207450009</v>
       </c>
       <c r="M2">
         <f>ABS(J2-D2)/D2*100</f>
-        <v>2.4962551020408013</v>
+        <v>1.8093750000000075</v>
       </c>
       <c r="N2">
         <f>ABS(K2-E2)/E2*100</f>
-        <v>0.73387905604719184</v>
+        <v>5.8035190615834398E-2</v>
       </c>
       <c r="O2">
-        <f>(ABS(L2-G2)/G2)*100</f>
-        <v>1.7495365635756437</v>
+        <f t="shared" ref="O2:O19" si="0">(ABS(L2-G2)/G2)*100</f>
+        <v>1.8684945750040829</v>
       </c>
       <c r="P2">
-        <f>(F2/C2)*100</f>
-        <v>91.520661157024804</v>
+        <f t="shared" ref="P2:P19" si="1">(F2/C2)*100</f>
+        <v>91.925333333333327</v>
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.25">
@@ -595,57 +595,57 @@
         <v>60</v>
       </c>
       <c r="B3">
-        <v>2.59</v>
+        <v>2.92</v>
       </c>
       <c r="C3">
         <f>A3*B3</f>
-        <v>155.39999999999998</v>
+        <v>175.2</v>
       </c>
       <c r="D3">
-        <v>20.94</v>
+        <v>22.96</v>
       </c>
       <c r="E3">
-        <v>6.91</v>
+        <v>7.13</v>
       </c>
       <c r="F3">
         <f>D3*E3</f>
-        <v>144.69540000000001</v>
+        <v>163.70480000000001</v>
       </c>
       <c r="G3">
         <f>D3/E3</f>
-        <v>3.0303907380607815</v>
+        <v>3.2201963534361853</v>
       </c>
       <c r="H3">
-        <v>35.786651999999997</v>
+        <v>36.469147</v>
       </c>
       <c r="I3">
-        <v>11.396839</v>
+        <v>10.580584999999999</v>
       </c>
       <c r="J3">
-        <v>21.406616</v>
+        <v>23.414888000000001</v>
       </c>
       <c r="K3">
-        <v>6.8172839999999999</v>
+        <v>6.793228</v>
       </c>
       <c r="L3">
         <f>J3/K3</f>
-        <v>3.140050495182539</v>
+        <v>3.4467984881414258</v>
       </c>
       <c r="M3">
-        <f t="shared" ref="M3:M19" si="0">ABS(J3-D3)/D3*100</f>
-        <v>2.2283476599808898</v>
+        <f t="shared" ref="M3:M19" si="2">ABS(J3-D3)/D3*100</f>
+        <v>1.9812195121951235</v>
       </c>
       <c r="N3">
-        <f t="shared" ref="N3:N19" si="1">ABS(K3-E3)/E3*100</f>
-        <v>1.3417655571635345</v>
+        <f t="shared" ref="N3:N19" si="3">ABS(K3-E3)/E3*100</f>
+        <v>4.7233099579242621</v>
       </c>
       <c r="O3">
-        <f>(ABS(L3-G3)/G3)*100</f>
-        <v>3.6186672479051767</v>
+        <f t="shared" si="0"/>
+        <v>7.0369042702454907</v>
       </c>
       <c r="P3">
-        <f>(F3/C3)*100</f>
-        <v>93.111583011583036</v>
+        <f t="shared" si="1"/>
+        <v>93.438812785388137</v>
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
@@ -653,57 +653,57 @@
         <v>60</v>
       </c>
       <c r="B4">
-        <v>2.75</v>
+        <v>2.88</v>
       </c>
       <c r="C4">
-        <f t="shared" ref="C4:C16" si="2">A2*B4</f>
-        <v>165</v>
+        <f t="shared" ref="C4:C16" si="4">A2*B4</f>
+        <v>172.79999999999998</v>
       </c>
       <c r="D4">
-        <v>22.15</v>
+        <v>23.63</v>
       </c>
       <c r="E4">
-        <v>6.94</v>
+        <v>6.86</v>
       </c>
       <c r="F4">
         <f>D4*E4</f>
-        <v>153.721</v>
+        <v>162.1018</v>
       </c>
       <c r="G4">
         <f>D4/E4</f>
-        <v>3.1916426512968297</v>
+        <v>3.444606413994169</v>
       </c>
       <c r="H4">
-        <v>35.784744000000003</v>
+        <v>36.011592999999998</v>
       </c>
       <c r="I4">
-        <v>10.764367999999999</v>
+        <v>10.135595</v>
       </c>
       <c r="J4">
-        <v>22.612379000000001</v>
+        <v>24.056635</v>
       </c>
       <c r="K4">
-        <v>6.8020040000000002</v>
+        <v>6.7708279999999998</v>
       </c>
       <c r="L4">
         <f>J4/K4</f>
-        <v>3.3243701415053564</v>
+        <v>3.5529827371187102</v>
       </c>
       <c r="M4">
-        <f t="shared" si="0"/>
-        <v>2.0874898419864656</v>
+        <f t="shared" si="2"/>
+        <v>1.805480321625057</v>
       </c>
       <c r="N4">
-        <f t="shared" si="1"/>
-        <v>1.9884149855907813</v>
+        <f t="shared" si="3"/>
+        <v>1.2998833819242051</v>
       </c>
       <c r="O4">
-        <f>(ABS(L4-G4)/G4)*100</f>
-        <v>4.1585949528089179</v>
+        <f t="shared" si="0"/>
+        <v>3.1462614330696246</v>
       </c>
       <c r="P4">
-        <f>(F4/C4)*100</f>
-        <v>93.164242424242431</v>
+        <f t="shared" si="1"/>
+        <v>93.808912037037047</v>
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
@@ -711,57 +711,57 @@
         <v>60</v>
       </c>
       <c r="B5">
-        <v>2.87</v>
+        <v>2.97</v>
       </c>
       <c r="C5">
-        <f t="shared" si="2"/>
-        <v>172.20000000000002</v>
+        <f t="shared" si="4"/>
+        <v>178.20000000000002</v>
       </c>
       <c r="D5">
-        <v>23.25</v>
+        <v>24.4</v>
       </c>
       <c r="E5" s="3">
-        <v>6.88</v>
+        <v>6.85</v>
       </c>
       <c r="F5">
         <f>D5*E5</f>
-        <v>159.96</v>
+        <v>167.14</v>
       </c>
       <c r="G5">
         <f>D5/E5</f>
-        <v>3.379360465116279</v>
+        <v>3.562043795620438</v>
       </c>
       <c r="H5">
-        <v>35.783969999999997</v>
+        <v>36.008194000000003</v>
       </c>
       <c r="I5">
-        <v>10.236521</v>
+        <v>9.7584610000000005</v>
       </c>
       <c r="J5">
-        <v>23.688374</v>
+        <v>24.833182999999998</v>
       </c>
       <c r="K5">
-        <v>6.7764009999999999</v>
+        <v>6.729959</v>
       </c>
       <c r="L5">
-        <f t="shared" ref="L5:L15" si="3">J5/K5</f>
-        <v>3.4957160888205996</v>
+        <f t="shared" ref="L5:L15" si="5">J5/K5</f>
+        <v>3.689945659401491</v>
       </c>
       <c r="M5">
-        <f t="shared" si="0"/>
-        <v>1.8854795698924713</v>
+        <f t="shared" si="2"/>
+        <v>1.7753401639344251</v>
       </c>
       <c r="N5">
-        <f t="shared" si="1"/>
-        <v>1.5057994186046511</v>
+        <f t="shared" si="3"/>
+        <v>1.7524233576642283</v>
       </c>
       <c r="O5">
-        <f>(ABS(L5-G5)/G5)*100</f>
-        <v>3.4431255530568854</v>
+        <f t="shared" si="0"/>
+        <v>3.5906875692631663</v>
       </c>
       <c r="P5">
-        <f>(F5/C5)*100</f>
-        <v>92.891986062717763</v>
+        <f t="shared" si="1"/>
+        <v>93.793490460157116</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
@@ -769,57 +769,57 @@
         <v>60</v>
       </c>
       <c r="B6">
-        <v>2.99</v>
+        <v>3.05</v>
       </c>
       <c r="C6">
-        <f t="shared" si="2"/>
-        <v>179.4</v>
+        <f t="shared" si="4"/>
+        <v>183</v>
       </c>
       <c r="D6">
-        <v>24.45</v>
+        <v>25.42</v>
       </c>
       <c r="E6" s="3">
-        <v>6.89</v>
+        <v>6.78</v>
       </c>
       <c r="F6">
         <f>D6*E6</f>
-        <v>168.4605</v>
+        <v>172.34760000000003</v>
       </c>
       <c r="G6">
         <f>D6/E6</f>
-        <v>3.5486211901306239</v>
+        <v>3.7492625368731565</v>
       </c>
       <c r="H6">
-        <v>35.786597999999998</v>
+        <v>36.011218999999997</v>
       </c>
       <c r="I6">
-        <v>9.6715370000000007</v>
+        <v>9.2680140000000009</v>
       </c>
       <c r="J6">
-        <v>24.878903999999999</v>
+        <v>25.833637</v>
       </c>
       <c r="K6">
-        <v>6.7236690000000001</v>
+        <v>6.6486640000000001</v>
       </c>
       <c r="L6">
-        <f t="shared" ref="L6" si="4">J6/K6</f>
-        <v>3.7001976153198495</v>
+        <f t="shared" ref="L6" si="6">J6/K6</f>
+        <v>3.8855380569690392</v>
       </c>
       <c r="M6">
-        <f t="shared" si="0"/>
-        <v>1.7542085889570525</v>
+        <f t="shared" si="2"/>
+        <v>1.6272108575924382</v>
       </c>
       <c r="N6">
-        <f t="shared" si="1"/>
-        <v>2.4140928882438253</v>
+        <f t="shared" si="3"/>
+        <v>1.9371091445427746</v>
       </c>
       <c r="O6">
-        <f>(ABS(L6-G6)/G6)*100</f>
-        <v>4.2714174623875829</v>
+        <f t="shared" si="0"/>
+        <v>3.634728663454307</v>
       </c>
       <c r="P6">
-        <f>(F6/C6)*100</f>
-        <v>93.90217391304347</v>
+        <f t="shared" si="1"/>
+        <v>94.179016393442637</v>
       </c>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
@@ -827,57 +827,57 @@
         <v>60</v>
       </c>
       <c r="B7">
-        <v>3.04</v>
+        <v>3.08</v>
       </c>
       <c r="C7">
+        <f t="shared" si="4"/>
+        <v>184.8</v>
+      </c>
+      <c r="D7">
+        <v>26.31</v>
+      </c>
+      <c r="E7">
+        <v>6.66</v>
+      </c>
+      <c r="F7">
+        <f t="shared" ref="F7" si="7">D7*E7</f>
+        <v>175.22459999999998</v>
+      </c>
+      <c r="G7">
+        <f t="shared" ref="G7" si="8">D7/E7</f>
+        <v>3.9504504504504503</v>
+      </c>
+      <c r="H7">
+        <v>36.012985</v>
+      </c>
+      <c r="I7">
+        <v>8.8198460000000001</v>
+      </c>
+      <c r="J7">
+        <v>26.700890000000001</v>
+      </c>
+      <c r="K7">
+        <v>6.5392450000000002</v>
+      </c>
+      <c r="L7">
+        <f t="shared" si="5"/>
+        <v>4.0831762688200239</v>
+      </c>
+      <c r="M7">
         <f t="shared" si="2"/>
-        <v>182.4</v>
-      </c>
-      <c r="D7">
-        <v>25.5</v>
-      </c>
-      <c r="E7">
-        <v>6.82</v>
-      </c>
-      <c r="F7">
-        <f t="shared" ref="F7" si="5">D7*E7</f>
-        <v>173.91</v>
-      </c>
-      <c r="G7">
-        <f t="shared" ref="G7" si="6">D7/E7</f>
-        <v>3.7390029325513194</v>
-      </c>
-      <c r="H7">
-        <v>35.785907999999999</v>
-      </c>
-      <c r="I7">
-        <v>9.1765559999999997</v>
-      </c>
-      <c r="J7">
-        <v>25.916357000000001</v>
-      </c>
-      <c r="K7">
-        <v>6.6457139999999999</v>
-      </c>
-      <c r="L7">
+        <v>1.4857088559483178</v>
+      </c>
+      <c r="N7">
         <f t="shared" si="3"/>
-        <v>3.8997099483968167</v>
-      </c>
-      <c r="M7">
-        <f t="shared" si="0"/>
-        <v>1.6327725490196134</v>
-      </c>
-      <c r="N7">
-        <f t="shared" si="1"/>
-        <v>2.5555131964809439</v>
+        <v>1.8131381381381373</v>
       </c>
       <c r="O7">
-        <f>(ABS(L7-G7)/G7)*100</f>
-        <v>4.2981248943776142</v>
+        <f t="shared" si="0"/>
+        <v>3.3597641594122409</v>
       </c>
       <c r="P7">
-        <f>(F7/C7)*100</f>
-        <v>95.34539473684211</v>
+        <f t="shared" si="1"/>
+        <v>94.818506493506476</v>
       </c>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.25">
@@ -888,54 +888,54 @@
         <v>3.11</v>
       </c>
       <c r="C8">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>186.6</v>
       </c>
       <c r="D8">
-        <v>26.27</v>
+        <v>27.05</v>
       </c>
       <c r="E8">
-        <v>6.72</v>
+        <v>6.56</v>
       </c>
       <c r="F8">
         <f>D8*E8</f>
-        <v>176.53439999999998</v>
+        <v>177.44800000000001</v>
       </c>
       <c r="G8">
-        <f t="shared" ref="G8:G12" si="7">D8/E8</f>
-        <v>3.9092261904761907</v>
+        <f t="shared" ref="G8:G12" si="9">D8/E8</f>
+        <v>4.1234756097560981</v>
       </c>
       <c r="H8">
-        <v>35.783023999999997</v>
+        <v>36.009430000000002</v>
       </c>
       <c r="I8">
-        <v>8.8042809999999996</v>
+        <v>8.417071</v>
       </c>
       <c r="J8">
-        <v>26.656096000000002</v>
+        <v>27.416253999999999</v>
       </c>
       <c r="K8">
-        <v>6.5586339999999996</v>
+        <v>6.4084479999999999</v>
       </c>
       <c r="L8">
+        <f t="shared" si="5"/>
+        <v>4.2781425393480603</v>
+      </c>
+      <c r="M8">
+        <f t="shared" si="2"/>
+        <v>1.353988909426979</v>
+      </c>
+      <c r="N8">
         <f t="shared" si="3"/>
-        <v>4.0642755793355754</v>
-      </c>
-      <c r="M8">
-        <f t="shared" si="0"/>
-        <v>1.4697221164826875</v>
-      </c>
-      <c r="N8">
-        <f t="shared" si="1"/>
-        <v>2.4012797619047639</v>
+        <v>2.3102439024390198</v>
       </c>
       <c r="O8">
-        <f>(ABS(L8-G8)/G8)*100</f>
-        <v>3.9662424557863152</v>
+        <f t="shared" si="0"/>
+        <v>3.7508874607145004</v>
       </c>
       <c r="P8">
-        <f>(F8/C8)*100</f>
-        <v>94.605787781350472</v>
+        <f t="shared" si="1"/>
+        <v>95.095391211146847</v>
       </c>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.25">
@@ -943,57 +943,57 @@
         <v>60</v>
       </c>
       <c r="B9">
-        <v>3.14</v>
+        <v>3.1</v>
       </c>
       <c r="C9">
-        <f t="shared" si="2"/>
-        <v>188.4</v>
+        <f t="shared" si="4"/>
+        <v>186</v>
       </c>
       <c r="D9">
-        <v>27.06</v>
+        <v>27.72</v>
       </c>
       <c r="E9">
-        <v>6.6</v>
+        <v>6.37</v>
       </c>
       <c r="F9">
         <f>D9*E9</f>
-        <v>178.59599999999998</v>
+        <v>176.57640000000001</v>
       </c>
       <c r="G9">
-        <f t="shared" ref="G9" si="8">D9/E9</f>
-        <v>4.0999999999999996</v>
+        <f t="shared" ref="G9" si="10">D9/E9</f>
+        <v>4.3516483516483513</v>
       </c>
       <c r="H9">
-        <v>35.787360999999997</v>
+        <v>36.009498999999998</v>
       </c>
       <c r="I9">
-        <v>8.3936209999999996</v>
+        <v>8.0225670000000004</v>
       </c>
       <c r="J9">
-        <v>27.416744000000001</v>
+        <v>28.057870999999999</v>
       </c>
       <c r="K9">
-        <v>6.4303650000000001</v>
+        <v>6.2510209999999997</v>
       </c>
       <c r="L9">
-        <f t="shared" ref="L9" si="9">J9/K9</f>
-        <v>4.2636372896406352</v>
+        <f t="shared" ref="L9" si="11">J9/K9</f>
+        <v>4.4885261143739559</v>
       </c>
       <c r="M9">
-        <f t="shared" si="0"/>
-        <v>1.3183444198078442</v>
+        <f t="shared" si="2"/>
+        <v>1.2188708513708508</v>
       </c>
       <c r="N9">
-        <f t="shared" si="1"/>
-        <v>2.5702272727272657</v>
+        <f t="shared" si="3"/>
+        <v>1.8678021978022037</v>
       </c>
       <c r="O9">
-        <f>(ABS(L9-G9)/G9)*100</f>
-        <v>3.9911534058691593</v>
+        <f t="shared" si="0"/>
+        <v>3.1454233353611158</v>
       </c>
       <c r="P9">
-        <f>(F9/C9)*100</f>
-        <v>94.796178343949038</v>
+        <f t="shared" si="1"/>
+        <v>94.933548387096778</v>
       </c>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
@@ -1001,57 +1001,57 @@
         <v>60</v>
       </c>
       <c r="B10">
-        <v>3.13</v>
+        <v>3.05</v>
       </c>
       <c r="C10">
-        <f t="shared" si="2"/>
-        <v>187.79999999999998</v>
+        <f t="shared" si="4"/>
+        <v>183</v>
       </c>
       <c r="D10">
-        <v>27.8</v>
+        <v>28.65</v>
       </c>
       <c r="E10">
-        <v>6.42</v>
+        <v>6.07</v>
       </c>
       <c r="F10">
         <f>D10*E10</f>
-        <v>178.476</v>
+        <v>173.90549999999999</v>
       </c>
       <c r="G10">
         <f>D10/E10</f>
-        <v>4.3302180685358254</v>
+        <v>4.7199341021416803</v>
       </c>
       <c r="H10">
-        <v>35.783805999999998</v>
+        <v>36.011665000000001</v>
       </c>
       <c r="I10">
-        <v>7.9662189999999997</v>
+        <v>7.3940039999999998</v>
       </c>
       <c r="J10">
-        <v>28.124404999999999</v>
+        <v>28.952494000000002</v>
       </c>
       <c r="K10">
-        <v>6.2610770000000002</v>
+        <v>5.9445969999999999</v>
       </c>
       <c r="L10">
+        <f t="shared" si="5"/>
+        <v>4.8703880178925507</v>
+      </c>
+      <c r="M10">
+        <f t="shared" si="2"/>
+        <v>1.0558254799302023</v>
+      </c>
+      <c r="N10">
         <f t="shared" si="3"/>
-        <v>4.4919436384507012</v>
-      </c>
-      <c r="M10">
-        <f t="shared" si="0"/>
-        <v>1.16692446043165</v>
-      </c>
-      <c r="N10">
-        <f t="shared" si="1"/>
-        <v>2.4754361370716462</v>
+        <v>2.0659472817133504</v>
       </c>
       <c r="O10">
-        <f>(ABS(L10-G10)/G10)*100</f>
-        <v>3.7348135210557665</v>
+        <f t="shared" si="0"/>
+        <v>3.1876274645995935</v>
       </c>
       <c r="P10">
-        <f>(F10/C10)*100</f>
-        <v>95.035143769968059</v>
+        <f t="shared" si="1"/>
+        <v>95.030327868852453</v>
       </c>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.25">
@@ -1059,57 +1059,57 @@
         <v>60</v>
       </c>
       <c r="B11">
-        <v>3.08</v>
+        <v>2.94</v>
       </c>
       <c r="C11">
-        <f t="shared" si="2"/>
-        <v>184.8</v>
+        <f t="shared" si="4"/>
+        <v>176.4</v>
       </c>
       <c r="D11">
-        <v>28.32</v>
+        <v>29.38</v>
       </c>
       <c r="E11">
-        <v>6.21</v>
+        <v>5.71</v>
       </c>
       <c r="F11">
         <f>D11*E11</f>
-        <v>175.8672</v>
+        <v>167.75979999999998</v>
       </c>
       <c r="G11">
-        <f t="shared" si="7"/>
-        <v>4.5603864734299515</v>
+        <f t="shared" si="9"/>
+        <v>5.1453590192644478</v>
       </c>
       <c r="H11">
-        <v>35.786223999999997</v>
+        <v>36.014778</v>
       </c>
       <c r="I11">
-        <v>7.6366769999999997</v>
+        <v>6.8235749999999999</v>
       </c>
       <c r="J11">
-        <v>28.616513999999999</v>
+        <v>29.632019</v>
       </c>
       <c r="K11">
-        <v>6.1066820000000002</v>
+        <v>5.6142589999999997</v>
       </c>
       <c r="L11">
+        <f t="shared" si="5"/>
+        <v>5.2779928749279295</v>
+      </c>
+      <c r="M11">
+        <f t="shared" si="2"/>
+        <v>0.85779101429544136</v>
+      </c>
+      <c r="N11">
         <f t="shared" si="3"/>
-        <v>4.6860986047742452</v>
-      </c>
-      <c r="M11">
-        <f t="shared" si="0"/>
-        <v>1.047012711864401</v>
-      </c>
-      <c r="N11">
-        <f t="shared" si="1"/>
-        <v>1.663735909822863</v>
+        <v>1.6767250437828425</v>
       </c>
       <c r="O11">
-        <f>(ABS(L11-G11)/G11)*100</f>
-        <v>2.7566113546894915</v>
+        <f t="shared" si="0"/>
+        <v>2.5777376304917636</v>
       </c>
       <c r="P11">
-        <f>(F11/C11)*100</f>
-        <v>95.166233766233759</v>
+        <f t="shared" si="1"/>
+        <v>95.101927437641706</v>
       </c>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.25">
@@ -1117,57 +1117,57 @@
         <v>60</v>
       </c>
       <c r="B12">
-        <v>3.02</v>
+        <v>2.79</v>
       </c>
       <c r="C12">
-        <f t="shared" si="2"/>
-        <v>181.2</v>
+        <f t="shared" si="4"/>
+        <v>167.4</v>
       </c>
       <c r="D12">
-        <v>29.08</v>
+        <v>30.09</v>
       </c>
       <c r="E12">
-        <v>5.93</v>
+        <v>5.32</v>
       </c>
       <c r="F12">
         <f>D12*E12</f>
-        <v>172.44439999999997</v>
+        <v>160.0788</v>
       </c>
       <c r="G12">
-        <f t="shared" si="7"/>
-        <v>4.9038785834738619</v>
+        <f t="shared" si="9"/>
+        <v>5.6560150375939848</v>
       </c>
       <c r="H12">
-        <v>35.786361999999997</v>
+        <v>36.012031999999998</v>
       </c>
       <c r="I12">
-        <v>7.083742</v>
+        <v>6.1987610000000002</v>
       </c>
       <c r="J12">
-        <v>29.345022</v>
+        <v>30.294250000000002</v>
       </c>
       <c r="K12">
-        <v>5.8087090000000003</v>
+        <v>5.2145570000000001</v>
       </c>
       <c r="L12">
+        <f t="shared" si="5"/>
+        <v>5.8095539084144638</v>
+      </c>
+      <c r="M12">
+        <f t="shared" si="2"/>
+        <v>0.6787969425058219</v>
+      </c>
+      <c r="N12">
         <f t="shared" si="3"/>
-        <v>5.0519008612757155</v>
-      </c>
-      <c r="M12">
-        <f t="shared" si="0"/>
-        <v>0.91135488308116186</v>
-      </c>
-      <c r="N12">
-        <f t="shared" si="1"/>
-        <v>2.0453794266441716</v>
+        <v>1.9820112781954919</v>
       </c>
       <c r="O12">
-        <f>(ABS(L12-G12)/G12)*100</f>
-        <v>3.0184735466471526</v>
+        <f t="shared" si="0"/>
+        <v>2.7146121394647666</v>
       </c>
       <c r="P12">
-        <f>(F12/C12)*100</f>
-        <v>95.16799116997791</v>
+        <f t="shared" si="1"/>
+        <v>95.626523297491033</v>
       </c>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.25">
@@ -1175,57 +1175,57 @@
         <v>60</v>
       </c>
       <c r="B13">
-        <v>2.89</v>
+        <v>2.59</v>
       </c>
       <c r="C13">
-        <f t="shared" si="2"/>
-        <v>173.4</v>
+        <f t="shared" si="4"/>
+        <v>155.39999999999998</v>
       </c>
       <c r="D13">
-        <v>29.86</v>
+        <v>30.52</v>
       </c>
       <c r="E13">
-        <v>5.53</v>
+        <v>4.8499999999999996</v>
       </c>
       <c r="F13">
-        <f t="shared" ref="F13:F14" si="10">D13*E13</f>
-        <v>165.1258</v>
+        <f t="shared" ref="F13:F14" si="12">D13*E13</f>
+        <v>148.02199999999999</v>
       </c>
       <c r="G13">
         <f>D13/E13</f>
-        <v>5.3996383363471967</v>
+        <v>6.2927835051546399</v>
       </c>
       <c r="H13">
-        <v>35.785271000000002</v>
+        <v>36.012630000000001</v>
       </c>
       <c r="I13">
-        <v>6.4420359999999999</v>
+        <v>5.7442089999999997</v>
       </c>
       <c r="J13">
-        <v>30.058085999999999</v>
+        <v>30.687252000000001</v>
       </c>
       <c r="K13">
-        <v>5.4110329999999998</v>
+        <v>4.8947830000000003</v>
       </c>
       <c r="L13">
+        <f t="shared" si="5"/>
+        <v>6.269379459722729</v>
+      </c>
+      <c r="M13">
+        <f t="shared" si="2"/>
+        <v>0.54800786369594134</v>
+      </c>
+      <c r="N13">
         <f t="shared" si="3"/>
-        <v>5.5549626106512378</v>
-      </c>
-      <c r="M13">
-        <f t="shared" si="0"/>
-        <v>0.66338245144005348</v>
-      </c>
-      <c r="N13">
-        <f t="shared" si="1"/>
-        <v>2.1513019891500993</v>
+        <v>0.9233608247422822</v>
       </c>
       <c r="O13">
-        <f>(ABS(L13-G13)/G13)*100</f>
-        <v>2.8765681075061855</v>
+        <f t="shared" si="0"/>
+        <v>0.37191880846909486</v>
       </c>
       <c r="P13">
-        <f>(F13/C13)*100</f>
-        <v>95.22825836216839</v>
+        <f t="shared" si="1"/>
+        <v>95.252252252252262</v>
       </c>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.25">
@@ -1233,57 +1233,57 @@
         <v>60</v>
       </c>
       <c r="B14">
-        <v>2.67</v>
+        <v>2.54</v>
       </c>
       <c r="C14">
-        <f t="shared" si="2"/>
-        <v>160.19999999999999</v>
+        <f t="shared" si="4"/>
+        <v>152.4</v>
       </c>
       <c r="D14">
-        <v>30.51</v>
+        <v>30.84</v>
       </c>
       <c r="E14">
-        <v>4.97</v>
+        <v>4.6900000000000004</v>
       </c>
       <c r="F14">
-        <f t="shared" si="10"/>
-        <v>151.63470000000001</v>
+        <f t="shared" si="12"/>
+        <v>144.6396</v>
       </c>
       <c r="G14">
         <f>D14/E14</f>
-        <v>6.1388329979879286</v>
+        <v>6.5756929637526644</v>
       </c>
       <c r="H14">
-        <v>36.241776000000002</v>
+        <v>36.012844000000001</v>
       </c>
       <c r="I14">
-        <v>5.8629949999999997</v>
+        <v>5.4196600000000004</v>
       </c>
       <c r="J14">
-        <v>30.656362999999999</v>
+        <v>30.963587</v>
       </c>
       <c r="K14">
-        <v>4.9594180000000003</v>
+        <v>4.6597850000000003</v>
       </c>
       <c r="L14">
+        <f t="shared" si="5"/>
+        <v>6.64485314236601</v>
+      </c>
+      <c r="M14">
+        <f t="shared" si="2"/>
+        <v>0.40073605706874371</v>
+      </c>
+      <c r="N14">
         <f t="shared" si="3"/>
-        <v>6.1814436693983037</v>
-      </c>
-      <c r="M14">
-        <f t="shared" si="0"/>
-        <v>0.47972140281873926</v>
-      </c>
-      <c r="N14">
-        <f t="shared" si="1"/>
-        <v>0.21291750503016951</v>
+        <v>0.64424307036247552</v>
       </c>
       <c r="O14">
-        <f>(ABS(L14-G14)/G14)*100</f>
-        <v>0.69411680403003695</v>
+        <f t="shared" si="0"/>
+        <v>1.051754986046014</v>
       </c>
       <c r="P14">
-        <f>(F14/C14)*100</f>
-        <v>94.653370786516859</v>
+        <f t="shared" si="1"/>
+        <v>94.907874015748035</v>
       </c>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.25">
@@ -1291,57 +1291,57 @@
         <v>60</v>
       </c>
       <c r="B15">
-        <v>2.46</v>
+        <v>2.36</v>
       </c>
       <c r="C15">
-        <f t="shared" si="2"/>
-        <v>147.6</v>
+        <f t="shared" si="4"/>
+        <v>141.6</v>
       </c>
       <c r="D15">
-        <v>31.18</v>
+        <v>31.33</v>
       </c>
       <c r="E15">
-        <v>4.5</v>
+        <v>4.3</v>
       </c>
       <c r="F15">
-        <f t="shared" ref="F15" si="11">D15*E15</f>
-        <v>140.31</v>
+        <f t="shared" ref="F15" si="13">D15*E15</f>
+        <v>134.71899999999999</v>
       </c>
       <c r="G15">
         <f>D15/E15</f>
-        <v>6.9288888888888884</v>
+        <v>7.286046511627907</v>
       </c>
       <c r="H15">
-        <v>35.787559999999999</v>
+        <v>36.013351</v>
       </c>
       <c r="I15">
-        <v>5.1022860000000003</v>
+        <v>4.8856070000000003</v>
       </c>
       <c r="J15">
-        <v>31.281769000000001</v>
+        <v>31.429310000000001</v>
       </c>
       <c r="K15">
-        <v>4.4598890000000004</v>
+        <v>4.2637309999999999</v>
       </c>
       <c r="L15">
+        <f t="shared" si="5"/>
+        <v>7.3713163424240413</v>
+      </c>
+      <c r="M15">
+        <f t="shared" si="2"/>
+        <v>0.31698052984360892</v>
+      </c>
+      <c r="N15">
         <f t="shared" si="3"/>
-        <v>7.0140241158468291</v>
-      </c>
-      <c r="M15">
-        <f t="shared" si="0"/>
-        <v>0.32639191789609007</v>
-      </c>
-      <c r="N15">
-        <f t="shared" si="1"/>
-        <v>0.89135555555554591</v>
+        <v>0.84346511627906717</v>
       </c>
       <c r="O15">
-        <f>(ABS(L15-G15)/G15)*100</f>
-        <v>1.2286995551979885</v>
+        <f t="shared" si="0"/>
+        <v>1.170316860591694</v>
       </c>
       <c r="P15">
-        <f>(F15/C15)*100</f>
-        <v>95.060975609756099</v>
+        <f t="shared" si="1"/>
+        <v>95.140536723163834</v>
       </c>
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.25">
@@ -1349,57 +1349,57 @@
         <v>60</v>
       </c>
       <c r="B16">
-        <v>2.14</v>
+        <v>2.02</v>
       </c>
       <c r="C16">
-        <f t="shared" si="2"/>
-        <v>128.4</v>
+        <f t="shared" si="4"/>
+        <v>121.2</v>
       </c>
       <c r="D16">
-        <v>31.69</v>
+        <v>31.87</v>
       </c>
       <c r="E16">
-        <v>3.84</v>
+        <v>3.58</v>
       </c>
       <c r="F16">
         <f>D16*E16</f>
-        <v>121.6896</v>
+        <v>114.0946</v>
       </c>
       <c r="G16">
-        <f t="shared" ref="G16:G19" si="12">D16/E16</f>
-        <v>8.2526041666666679</v>
+        <f t="shared" ref="G16:G19" si="14">D16/E16</f>
+        <v>8.9022346368715084</v>
       </c>
       <c r="H16">
-        <v>35.788845000000002</v>
+        <v>36.014510999999999</v>
       </c>
       <c r="I16">
-        <v>4.3173950000000003</v>
+        <v>4.0447050000000004</v>
       </c>
       <c r="J16">
-        <v>31.720699</v>
+        <v>31.895897000000001</v>
       </c>
       <c r="K16">
-        <v>3.8266330000000002</v>
+        <v>3.5821529999999999</v>
       </c>
       <c r="L16">
-        <f t="shared" ref="L16:L19" si="13">J16/K16</f>
-        <v>8.2894542016441086</v>
+        <f t="shared" ref="L16:L19" si="15">J16/K16</f>
+        <v>8.9041135317224036</v>
       </c>
       <c r="M16">
-        <f t="shared" si="0"/>
-        <v>9.6872830545908728E-2</v>
+        <f t="shared" si="2"/>
+        <v>8.1258236586132723E-2</v>
       </c>
       <c r="N16">
-        <f t="shared" si="1"/>
-        <v>0.34809895833332516</v>
+        <f t="shared" si="3"/>
+        <v>6.0139664804465059E-2</v>
       </c>
       <c r="O16">
-        <f>(ABS(L16-G16)/G16)*100</f>
-        <v>0.44652614172727212</v>
+        <f t="shared" si="0"/>
+        <v>2.1105878776921376E-2</v>
       </c>
       <c r="P16">
-        <f>(F16/C16)*100</f>
-        <v>94.773831775700927</v>
+        <f t="shared" si="1"/>
+        <v>94.137458745874582</v>
       </c>
     </row>
     <row r="17" spans="1:16" x14ac:dyDescent="0.25">
@@ -1407,57 +1407,57 @@
         <v>60</v>
       </c>
       <c r="B17">
-        <v>1.39</v>
+        <v>1.53</v>
       </c>
       <c r="C17">
-        <f t="shared" ref="C17:C19" si="14">A15*B17</f>
-        <v>83.399999999999991</v>
+        <f t="shared" ref="C17:C19" si="16">A15*B17</f>
+        <v>91.8</v>
       </c>
       <c r="D17">
-        <v>31.84</v>
+        <v>32.56</v>
       </c>
       <c r="E17">
-        <v>2.36</v>
+        <v>2.63</v>
       </c>
       <c r="F17">
-        <f t="shared" ref="F17:F19" si="15">D17*E17</f>
-        <v>75.142399999999995</v>
+        <f t="shared" ref="F17:F19" si="17">D17*E17</f>
+        <v>85.632800000000003</v>
       </c>
       <c r="G17">
-        <f t="shared" si="12"/>
-        <v>13.491525423728815</v>
+        <f t="shared" si="14"/>
+        <v>12.380228136882131</v>
       </c>
       <c r="H17">
-        <v>35.790173000000003</v>
+        <v>36.019165000000001</v>
       </c>
       <c r="I17">
-        <v>2.6143000000000001</v>
+        <v>2.9405770000000002</v>
       </c>
       <c r="J17">
-        <v>32.716628999999998</v>
+        <v>32.502819000000002</v>
       </c>
       <c r="K17">
-        <v>2.3897919999999999</v>
+        <v>2.653505</v>
       </c>
       <c r="L17">
-        <f t="shared" si="13"/>
-        <v>13.690157553460718</v>
+        <f t="shared" si="15"/>
+        <v>12.249013663060746</v>
       </c>
       <c r="M17">
-        <f t="shared" si="0"/>
-        <v>2.753231783919591</v>
+        <f t="shared" si="2"/>
+        <v>0.17561732186732162</v>
       </c>
       <c r="N17">
-        <f t="shared" si="1"/>
-        <v>1.2623728813559341</v>
+        <f t="shared" si="3"/>
+        <v>0.89372623574144905</v>
       </c>
       <c r="O17">
-        <f>(ABS(L17-G17)/G17)*100</f>
-        <v>1.4722733233897358</v>
+        <f t="shared" si="0"/>
+        <v>1.059871210535148</v>
       </c>
       <c r="P17">
-        <f>(F17/C17)*100</f>
-        <v>90.098800959232619</v>
+        <f t="shared" si="1"/>
+        <v>93.281917211328974</v>
       </c>
     </row>
     <row r="18" spans="1:16" x14ac:dyDescent="0.25">
@@ -1465,57 +1465,57 @@
         <v>60</v>
       </c>
       <c r="B18">
-        <v>0.68</v>
+        <v>0.81</v>
       </c>
       <c r="C18">
+        <f t="shared" si="16"/>
+        <v>48.6</v>
+      </c>
+      <c r="D18">
+        <v>33.51</v>
+      </c>
+      <c r="E18">
+        <v>1.31</v>
+      </c>
+      <c r="F18">
+        <f t="shared" si="17"/>
+        <v>43.898099999999999</v>
+      </c>
+      <c r="G18">
         <f t="shared" si="14"/>
-        <v>40.800000000000004</v>
-      </c>
-      <c r="D18">
-        <v>33.770000000000003</v>
-      </c>
-      <c r="E18">
-        <v>1.05</v>
-      </c>
-      <c r="F18">
+        <v>25.580152671755723</v>
+      </c>
+      <c r="H18">
+        <v>36.026187999999998</v>
+      </c>
+      <c r="I18">
+        <v>1.5182819999999999</v>
+      </c>
+      <c r="J18">
+        <v>33.319305</v>
+      </c>
+      <c r="K18">
+        <v>1.404204</v>
+      </c>
+      <c r="L18">
         <f t="shared" si="15"/>
-        <v>35.458500000000008</v>
-      </c>
-      <c r="G18">
-        <f t="shared" si="12"/>
-        <v>32.161904761904765</v>
-      </c>
-      <c r="H18">
-        <v>35.804442999999999</v>
-      </c>
-      <c r="I18">
-        <v>1.283223</v>
-      </c>
-      <c r="J18">
-        <v>33.539886000000003</v>
-      </c>
-      <c r="K18">
-        <v>1.202061</v>
-      </c>
-      <c r="L18">
-        <f t="shared" si="13"/>
-        <v>27.901983343607355</v>
+        <v>23.728251023355579</v>
       </c>
       <c r="M18">
-        <f t="shared" si="0"/>
-        <v>0.68141545750666377</v>
+        <f t="shared" si="2"/>
+        <v>0.56906893464636843</v>
       </c>
       <c r="N18">
-        <f t="shared" si="1"/>
-        <v>14.482000000000001</v>
+        <f t="shared" si="3"/>
+        <v>7.191145038167936</v>
       </c>
       <c r="O18">
-        <f>(ABS(L18-G18)/G18)*100</f>
-        <v>13.24523982591732</v>
+        <f t="shared" si="0"/>
+        <v>7.2396035792425817</v>
       </c>
       <c r="P18">
-        <f>(F18/C18)*100</f>
-        <v>86.908088235294116</v>
+        <f t="shared" si="1"/>
+        <v>90.325308641975312</v>
       </c>
     </row>
     <row r="19" spans="1:16" x14ac:dyDescent="0.25">
@@ -1526,54 +1526,54 @@
         <v>0.15</v>
       </c>
       <c r="C19">
-        <f t="shared" si="14"/>
+        <f t="shared" si="16"/>
         <v>9</v>
       </c>
       <c r="D19">
-        <v>34.51</v>
+        <v>34.35</v>
       </c>
       <c r="E19">
         <v>0.08</v>
       </c>
       <c r="F19">
+        <f t="shared" si="17"/>
+        <v>2.7480000000000002</v>
+      </c>
+      <c r="G19">
+        <f t="shared" si="14"/>
+        <v>429.375</v>
+      </c>
+      <c r="H19">
+        <v>36.040680000000002</v>
+      </c>
+      <c r="I19">
+        <v>0.27150299999999999</v>
+      </c>
+      <c r="J19">
+        <v>34.069290000000002</v>
+      </c>
+      <c r="K19">
+        <v>0.25665199999999999</v>
+      </c>
+      <c r="L19">
         <f t="shared" si="15"/>
-        <v>2.7607999999999997</v>
-      </c>
-      <c r="G19">
-        <f t="shared" si="12"/>
-        <v>431.37499999999994</v>
-      </c>
-      <c r="H19">
-        <v>35.815018000000002</v>
-      </c>
-      <c r="I19">
-        <v>0.28751399999999999</v>
-      </c>
-      <c r="J19">
-        <v>34.182873000000001</v>
-      </c>
-      <c r="K19">
-        <v>0.27441199999999999</v>
-      </c>
-      <c r="L19">
-        <f t="shared" si="13"/>
-        <v>124.56770476509774</v>
+        <v>132.74507893957579</v>
       </c>
       <c r="M19">
-        <f t="shared" si="0"/>
-        <v>0.94791944363951697</v>
+        <f t="shared" si="2"/>
+        <v>0.81720524017466989</v>
       </c>
       <c r="N19">
-        <f t="shared" si="1"/>
-        <v>243.01499999999999</v>
+        <f t="shared" si="3"/>
+        <v>220.815</v>
       </c>
       <c r="O19">
-        <f>(ABS(L19-G19)/G19)*100</f>
-        <v>71.12310524135664</v>
+        <f t="shared" si="0"/>
+        <v>69.084115530812042</v>
       </c>
       <c r="P19">
-        <f>(F19/C19)*100</f>
-        <v>30.675555555555551</v>
+        <f t="shared" si="1"/>
+        <v>30.533333333333335</v>
       </c>
     </row>
   </sheetData>

</xml_diff>